<commit_message>
Fix Stars 2027 PP1 measure weights and polish contract reports.
Use stars-year workbook weights (Call Center D=2, HOS physical/mental=3), match mistitled Part C/D twins, and surface Part C/D ratings plus scenario acronyms in the report.

Co-authored-by: Cursor <cursoragent@cursor.com>
</commit_message>
<xml_diff>
--- a/data/Stars 2016-2028 Cut Points 07.2026_with_weights.xlsx
+++ b/data/Stars 2016-2028 Cut Points 07.2026_with_weights.xlsx
@@ -13388,7 +13388,7 @@
         <v>89</v>
       </c>
       <c r="I448">
-        <v>1</v>
+        <v>3</v>
       </c>
     </row>
     <row r="449">
@@ -13417,7 +13417,7 @@
         <v>76</v>
       </c>
       <c r="I449">
-        <v>1</v>
+        <v>3</v>
       </c>
     </row>
     <row r="450">

</xml_diff>